<commit_message>
Enhance BLE compatibility with Home Assistant integration by updating advertisement parameters and security settings
</commit_message>
<xml_diff>
--- a/docs/bill_of_materials.xlsx
+++ b/docs/bill_of_materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kok/CLionProjects/esp32-light-switch/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C1978F-CB28-C94E-9FFA-AD62C627E7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE372F0-9D3B-084F-BCE6-A033D01A6682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4140" yWindow="2700" windowWidth="28040" windowHeight="17180" xr2:uid="{3925CBBA-9425-4243-AAD1-1C53B1364004}"/>
+    <workbookView xWindow="4340" yWindow="3060" windowWidth="28040" windowHeight="17180" xr2:uid="{3925CBBA-9425-4243-AAD1-1C53B1364004}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,9 +59,6 @@
     <t>ESP32-WROOM-32E</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005010001114193.html?spm=a2g0o.productlist.main.2.1e411c60tBxnrI&amp;algo_pvid=7f81ab6e-c626-4516-930a-f26c57c35cb3&amp;algo_exp_id=7f81ab6e-c626-4516-930a-f26c57c35cb3-1&amp;pdp_ext_f=%7B%22order%22%3A%2287%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21BGN%2111.06%2111.28%21%21%2145.72%2146.63%21%40211b431017717531002058647eb05b%2112000050806262041%21sea%21BG%213190334324%21X%211%210%21n_tag%3A-29919%3Bd%3A74fd2ea5%3Bm03_new_user%3A-29895&amp;curPageLogUid=aFv157UnmCcQ&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010001114193%7C_p_origin_prod%3A</t>
-  </si>
-  <si>
     <t>https://tpetrov.com/ltv817s-lit-247331</t>
   </si>
   <si>
@@ -227,7 +224,10 @@
     <t>WS2812B LED</t>
   </si>
   <si>
-    <t>C1, C3, C4, C6, C8, C9</t>
+    <t>C1, C4, C6, C8, C9</t>
+  </si>
+  <si>
+    <t>https://bulcomp-eng.com/m/index.php?p=10&amp;idprod=19925</t>
   </si>
 </sst>
 </file>
@@ -699,7 +699,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
@@ -715,31 +715,31 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="4">
         <v>1</v>
       </c>
       <c r="D3" s="5">
-        <v>3</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="E3" s="5">
         <f t="shared" ref="E3:E22" si="0">C3*D3</f>
-        <v>3</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="4">
         <v>1</v>
@@ -752,15 +752,15 @@
         <v>0.26</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4">
         <v>1</v>
@@ -773,15 +773,15 @@
         <v>1.07</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="C6" s="4">
         <v>1</v>
@@ -794,15 +794,15 @@
         <v>0.26</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="4">
         <v>1</v>
@@ -818,10 +818,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4">
         <v>1</v>
@@ -834,36 +834,36 @@
         <v>0.64</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="5">
         <v>0.06</v>
       </c>
       <c r="E9" s="5">
         <f t="shared" si="0"/>
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="C10" s="4">
         <v>1</v>
@@ -876,15 +876,15 @@
         <v>0.08</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="C11" s="4">
         <v>1</v>
@@ -897,15 +897,15 @@
         <v>0.1</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="C12" s="4">
         <v>1</v>
@@ -918,15 +918,15 @@
         <v>0.08</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="4">
         <v>3</v>
@@ -935,19 +935,19 @@
         <v>0.03</v>
       </c>
       <c r="E13" s="5">
-        <f>C13*D13</f>
+        <f t="shared" ref="E13:E21" si="1">C13*D13</f>
         <v>0.09</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C14" s="4">
         <v>2</v>
@@ -956,19 +956,19 @@
         <v>0.06</v>
       </c>
       <c r="E14" s="5">
-        <f>C14*D14</f>
+        <f t="shared" si="1"/>
         <v>0.12</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" s="4">
         <v>2</v>
@@ -977,19 +977,19 @@
         <v>0.09</v>
       </c>
       <c r="E15" s="5">
-        <f>C15*D15</f>
+        <f t="shared" si="1"/>
         <v>0.18</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16" s="4">
         <v>1</v>
@@ -998,19 +998,19 @@
         <v>0.97</v>
       </c>
       <c r="E16" s="5">
-        <f>C16*D16</f>
+        <f t="shared" si="1"/>
         <v>0.97</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" s="4">
         <v>1</v>
@@ -1019,19 +1019,19 @@
         <v>0.36</v>
       </c>
       <c r="E17" s="5">
-        <f>C17*D17</f>
+        <f t="shared" si="1"/>
         <v>0.36</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" s="4">
         <v>1</v>
@@ -1040,19 +1040,19 @@
         <v>0.1</v>
       </c>
       <c r="E18" s="5">
-        <f>C18*D18</f>
+        <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C19" s="4">
         <v>1</v>
@@ -1061,19 +1061,19 @@
         <v>0.26</v>
       </c>
       <c r="E19" s="5">
-        <f>C19*D19</f>
+        <f t="shared" si="1"/>
         <v>0.26</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C20" s="4">
         <v>1</v>
@@ -1082,19 +1082,19 @@
         <v>0.1</v>
       </c>
       <c r="E20" s="5">
-        <f>C20*D20</f>
+        <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C21" s="4">
         <v>1</v>
@@ -1103,19 +1103,19 @@
         <v>0.51</v>
       </c>
       <c r="E21" s="5">
-        <f>C21*D21</f>
+        <f t="shared" si="1"/>
         <v>0.51</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" s="4">
         <v>1</v>
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1138,7 +1138,7 @@
       <c r="D23" s="9"/>
       <c r="E23" s="9">
         <f>SUM(E2:E22)</f>
-        <v>8.5399999999999991</v>
+        <v>9.8299999999999965</v>
       </c>
       <c r="F23" s="7"/>
     </row>
@@ -1153,6 +1153,8 @@
     <hyperlink ref="F15" r:id="rId6" xr:uid="{37D7826B-6518-3A48-83DA-8658A7B84E20}"/>
     <hyperlink ref="F18" r:id="rId7" xr:uid="{30B50112-4124-4047-8A14-8503A3EA9C9F}"/>
     <hyperlink ref="F17" r:id="rId8" xr:uid="{159B2F44-44FE-CD4C-B025-8D97CFABE804}"/>
+    <hyperlink ref="F19" r:id="rId9" xr:uid="{65938BED-2C28-574C-9EE1-D7D3370B14F8}"/>
+    <hyperlink ref="F3" r:id="rId10" xr:uid="{CC3186DF-4FFD-B244-A59D-C7603D291DBC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>